<commit_message>
Restore drawings stripped by openpyxl save
openpyxl rebuilds the xlsx from its object model, silently dropping parts it
does not understand. Writing press-release links removed xl/drawings/drawing1.xml
-- two arrow connectors on the Model sheet -- from 27 models.

Adds xlsx_safe.save_workbook(), which saves through openpyxl and then re-injects
any dropped part along with its content-type, relationship, and the owning
sheet's <drawing> element. Restores the drawing in the 27 affected models;
all 693 existing links verified intact.

sharedStrings is not restored: openpyxl inlines strings, so its absence is
correct rather than damage.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AEP.xlsx
+++ b/AEP.xlsx
@@ -129,6 +129,117 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="3" name="Straight Arrow Connector 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6034B925-50E7-A3CC-FAE6-8C775CCD7564}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="23139400" y="63500"/>
+          <a:ext cx="0" cy="8267700"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>63500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>38</xdr:col>
+      <xdr:colOff>25400</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="4" name="Straight Arrow Connector 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7CEFFD1E-95F6-BC41-B05B-5DB09CB2C836}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="31394400" y="63500"/>
+          <a:ext cx="0" cy="8267700"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -698,5 +809,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId27"/>
 </worksheet>
 </file>
</xml_diff>